<commit_message>
Hotline-Excel: alle 0137-Nummern Frage 1-5 (statt nur 1+5)
</commit_message>
<xml_diff>
--- a/docs/Hotline-Zuordnung.xlsx
+++ b/docs/Hotline-Zuordnung.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referenz 0800" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Zuordnung'!$A$1:$I$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Zuordnung'!$A$1:$L$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -482,10 +482,13 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,30 +509,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>0137 Frage2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>0137 Frage3</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>0137 Frage4</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>0137 Frage5</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>0137-Status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>0137-Korrektur</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>0800 (Service)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>0800-Status</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>0800-Korrektur</t>
         </is>
@@ -553,26 +571,41 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>01378 005562</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>01378 005563</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>01378 005564</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>01378 005565</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>0800-2001199</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -592,26 +625,41 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>01379 441292</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>01379 441293</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>01379 441294</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>01379 441295</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>0800-7779872</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -631,26 +679,41 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>01379 441282</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>01379 441283</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>01379 441284</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>01379 441285</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>0800-7779872</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -670,26 +733,41 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>01379 441272</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>01379 441273</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>01379 441274</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>01379 441275</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>0800-7779872</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -712,23 +790,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -751,23 +844,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -790,23 +898,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -826,26 +949,41 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>01378 405282</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>01378 405283</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>01378 405284</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
           <t>01378 405285</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -865,26 +1003,41 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>01378 405282</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>01378 405283</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>01378 405284</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
           <t>01378 405285</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>BITTE PRÜFEN</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -904,26 +1057,41 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>01378 407282</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>01378 407283</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>01378 407284</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
           <t>01378 407285</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -943,26 +1111,41 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>01378 407282</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>01378 407283</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>01378 407284</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
           <t>01378 407285</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -985,23 +1168,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1021,26 +1219,41 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>01378 404382</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>01378 404383</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>01378 404384</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
           <t>01378 404385</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1060,26 +1273,41 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>01378 406282</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>01378 406283</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>01378 406284</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
           <t>01378 406285</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1102,23 +1330,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1138,26 +1381,41 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>01378 403892</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>01378 403893</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>01378 403894</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
           <t>01378 403895</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1177,26 +1435,41 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>01378 403792</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>01378 403793</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>01378 403794</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
           <t>01378 403795</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1219,23 +1492,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1258,23 +1546,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1297,23 +1600,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1336,23 +1654,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="K22" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1375,23 +1708,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1414,23 +1762,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="K24" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1453,23 +1816,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1492,23 +1870,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1531,23 +1924,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1567,26 +1975,41 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
+          <t>01379 441272</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>01379 441273</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>01379 441274</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
           <t>01379 441275</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>BITTE PRÜFEN</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1606,26 +2029,41 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
+          <t>01378 406182</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>01378 406183</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>01378 406184</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
           <t>01378 406185</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1645,26 +2083,41 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
+          <t>01378 406582</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>01378 406583</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>01378 406584</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
           <t>01378 406585</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr"/>
+      <c r="L30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1687,23 +2140,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1726,23 +2194,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>0800-2223384</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr"/>
+      <c r="L32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1765,23 +2248,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>0800-7779878</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1801,26 +2299,41 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
+          <t>01378 220272</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>01378 220273</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>01378 220274</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
           <t>01378 220275</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>0800-1011326</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="K34" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr"/>
+      <c r="L34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1843,23 +2356,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>0800-1088100</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="K35" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1879,26 +2407,41 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
+          <t>01378 806372</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>01378 806373</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>01378 806374</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
           <t>01378 806375</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="I36" s="4" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>0800-2223385</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="K36" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr"/>
+      <c r="L36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1918,26 +2461,41 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
+          <t>01378 806172</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>01378 806173</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>01378 806174</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
           <t>01378 806175</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>0800-2223385</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
+      <c r="K37" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1957,26 +2515,41 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
+          <t>01378 806272</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>01378 806273</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>01378 806274</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
           <t>01378 806275</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="I38" s="4" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>0800-2223385</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="K38" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr"/>
+      <c r="L38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1999,23 +2572,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>0800-2223365</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="K39" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2035,26 +2623,41 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
+          <t>01378 805772</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>01378 805773</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>01378 805774</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
           <t>01378 805775</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr"/>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="I40" s="4" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>0800-2223365</t>
         </is>
       </c>
-      <c r="H40" s="3" t="inlineStr">
+      <c r="K40" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr"/>
+      <c r="L40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2074,26 +2677,41 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
+          <t>01378 403882</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>01378 403883</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>01378 403884</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
           <t>01378 403885</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>BITTE PRÜFEN</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>0800-2223365</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr">
+      <c r="K41" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr"/>
+      <c r="L41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2113,26 +2731,41 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
+          <t>01378 408172</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>01378 408173</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>01378 408174</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
           <t>01378 408175</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="H42" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="I42" s="4" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>0800-2224449</t>
         </is>
       </c>
-      <c r="H42" s="3" t="inlineStr">
+      <c r="K42" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I42" s="4" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2152,26 +2785,41 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
+          <t>01378 408272</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>01378 408273</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>01378 408274</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
           <t>01378 408275</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
         <is>
           <t>0800-2224449</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr">
+      <c r="K43" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2194,23 +2842,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>0800-2224449</t>
         </is>
       </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="K44" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr"/>
+      <c r="L44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2230,26 +2893,41 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
+          <t>01378 408572</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>01378 408573</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>01378 408574</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
           <t>01378 408575</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>0800-2224449</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr">
+      <c r="K45" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2269,26 +2947,41 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
+          <t>01378 408172</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>01378 408173</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>01378 408174</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
           <t>01378 408175</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="H46" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="I46" s="4" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>0800-2224449</t>
         </is>
       </c>
-      <c r="H46" s="3" t="inlineStr">
+      <c r="K46" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I46" s="4" t="inlineStr"/>
+      <c r="L46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2308,26 +3001,41 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
+          <t>01378 408472</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>01378 408473</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>01378 408474</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
           <t>01378 408475</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>0800-2224449</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr">
+      <c r="K47" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2350,23 +3058,38 @@
           <t>(Platzhalter)</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>(Platzhalter)</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
         <is>
           <t>OFFEN – manuell</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="I48" s="4" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>0800-2224449</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr">
+      <c r="K48" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I48" s="4" t="inlineStr"/>
+      <c r="L48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2386,29 +3109,44 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
+          <t>01378 803872</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>01378 803873</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>01378 803874</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
           <t>01378 803875</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr">
         <is>
           <t>gekoppelt</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>0800-7779889</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr">
+      <c r="K49" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I49"/>
+  <autoFilter ref="A1:L49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2423,11 +3161,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>

</xml_diff>